<commit_message>
Actualización: Unificación de tarjeta informativa y módulos de calendario
</commit_message>
<xml_diff>
--- a/datos_asistencias.xlsx
+++ b/datos_asistencias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,188 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AGUIRRE, ERIKA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-08-29 14:38:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AGUIRRE, ERIKA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C4" t="n">
+        <v>8</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-08-04</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-08-29 14:58:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AGUIRRE, ERIKA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C5" t="n">
+        <v>8</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Se retiró</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Se sentía mal - 12hs.</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-08-30 17:23:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AGUIRRE, ERIKA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-08-30 17:31:03</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>AGUIRRE, ERIKA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C7" t="n">
+        <v>8</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-08-06</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2026-08-30 17:31:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>AGUIRRE, ERIKA ALEJANDRA</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C8" t="n">
+        <v>8</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-08-07</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Se retiró</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Por falta de huevos</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-08-30 17:31:19</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Se supone que con la lista de asesores del selector de asistencias, arreglado
</commit_message>
<xml_diff>
--- a/datos_asistencias.xlsx
+++ b/datos_asistencias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,7 +456,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AGUIRRE, ERIKA ALEJANDRA</t>
+          <t>AGUIRRE ERIKA</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -472,195 +472,17 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Ausente</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>Se retiró</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>12hs.</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-08-29 12:01:25</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>AGUIRRE, ERIKA ALEJANDRA</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C3" t="n">
-        <v>8</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>2026-08-29 14:38:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>AGUIRRE, ERIKA ALEJANDRA</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C4" t="n">
-        <v>8</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>2026-08-04</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>2026-08-29 14:58:17</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>AGUIRRE, ERIKA ALEJANDRA</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C5" t="n">
-        <v>8</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>2026-08-03</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Se retiró</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>Se sentía mal - 12hs.</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>2026-08-30 17:23:29</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>AGUIRRE, ERIKA ALEJANDRA</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C6" t="n">
-        <v>8</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>2026-08-30 17:31:03</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>AGUIRRE, ERIKA ALEJANDRA</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Presente</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>2026-08-30 17:31:07</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>AGUIRRE, ERIKA ALEJANDRA</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C8" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>2026-08-07</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Se retiró</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Por falta de huevos</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>2026-08-30 17:31:19</t>
+          <t>2026-08-30 22:36:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agregada navegacion por meses en el panel del asesor
</commit_message>
<xml_diff>
--- a/datos_asistencias.xlsx
+++ b/datos_asistencias.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -483,6 +483,64 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-08-30 22:36:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AGUIRRE ERIKA</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C3" t="n">
+        <v>9</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2026-08-31 16:30:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>AGUIRRE ERIKA</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C4" t="n">
+        <v>9</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Presente</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-08-31 16:30:41</t>
         </is>
       </c>
     </row>

</xml_diff>